<commit_message>
Replace remote repository with latest local code
</commit_message>
<xml_diff>
--- a/customer_vertical_mapping.xlsx
+++ b/customer_vertical_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmounika/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08CA848-E847-1C43-AE55-17732B069101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE9012DA-4768-064E-8985-D875BD7245CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1573,9 +1573,6 @@
     <t>Ashit Sharma</t>
   </si>
   <si>
-    <t>Amit Raj</t>
-  </si>
-  <si>
     <t>Somasundaram Venugopal</t>
   </si>
   <si>
@@ -1588,13 +1585,16 @@
     <t xml:space="preserve">Siddiq Mohamed </t>
   </si>
   <si>
-    <t xml:space="preserve">Bala Shekar </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arun Kaliappan / Jyaram O P / Ankur Tyagi </t>
-  </si>
-  <si>
-    <t>Arun Kaliappan</t>
+    <t xml:space="preserve">Bala Sekar </t>
+  </si>
+  <si>
+    <t>Amit Rai</t>
+  </si>
+  <si>
+    <t>B Arun Kaliappan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B Arun Kaliappan / Jyaram O P / Ankur Tyagi </t>
   </si>
 </sst>
 </file>
@@ -2004,7 +2004,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2015,7 +2015,7 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2026,7 +2026,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -2037,7 +2037,7 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2048,7 +2048,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2059,7 +2059,7 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -2070,7 +2070,7 @@
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2081,7 +2081,7 @@
         <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2092,7 +2092,7 @@
         <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2103,7 +2103,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -2114,7 +2114,7 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -2224,7 +2224,7 @@
         <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -2235,7 +2235,7 @@
         <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -2246,7 +2246,7 @@
         <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -2257,7 +2257,7 @@
         <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -2268,7 +2268,7 @@
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -2279,7 +2279,7 @@
         <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -2290,7 +2290,7 @@
         <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -2301,7 +2301,7 @@
         <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -2312,7 +2312,7 @@
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -2323,7 +2323,7 @@
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -2334,7 +2334,7 @@
         <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -2345,7 +2345,7 @@
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -2356,7 +2356,7 @@
         <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -2367,7 +2367,7 @@
         <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -2378,7 +2378,7 @@
         <v>42</v>
       </c>
       <c r="C37" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -2389,7 +2389,7 @@
         <v>43</v>
       </c>
       <c r="C38" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -2400,7 +2400,7 @@
         <v>44</v>
       </c>
       <c r="C39" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -2411,7 +2411,7 @@
         <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -2422,7 +2422,7 @@
         <v>46</v>
       </c>
       <c r="C41" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -2433,7 +2433,7 @@
         <v>47</v>
       </c>
       <c r="C42" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -2444,7 +2444,7 @@
         <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -2455,7 +2455,7 @@
         <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -2466,7 +2466,7 @@
         <v>50</v>
       </c>
       <c r="C45" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -2477,7 +2477,7 @@
         <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -2488,7 +2488,7 @@
         <v>52</v>
       </c>
       <c r="C47" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -2499,7 +2499,7 @@
         <v>53</v>
       </c>
       <c r="C48" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -2510,7 +2510,7 @@
         <v>54</v>
       </c>
       <c r="C49" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -2521,7 +2521,7 @@
         <v>55</v>
       </c>
       <c r="C50" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -2532,7 +2532,7 @@
         <v>56</v>
       </c>
       <c r="C51" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -2543,7 +2543,7 @@
         <v>57</v>
       </c>
       <c r="C52" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -2554,7 +2554,7 @@
         <v>58</v>
       </c>
       <c r="C53" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -2565,7 +2565,7 @@
         <v>59</v>
       </c>
       <c r="C54" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -2576,7 +2576,7 @@
         <v>60</v>
       </c>
       <c r="C55" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -2587,7 +2587,7 @@
         <v>61</v>
       </c>
       <c r="C56" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -2598,7 +2598,7 @@
         <v>62</v>
       </c>
       <c r="C57" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -2609,7 +2609,7 @@
         <v>63</v>
       </c>
       <c r="C58" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -2620,7 +2620,7 @@
         <v>64</v>
       </c>
       <c r="C59" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -2631,7 +2631,7 @@
         <v>65</v>
       </c>
       <c r="C60" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
@@ -2642,7 +2642,7 @@
         <v>66</v>
       </c>
       <c r="C61" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -2653,7 +2653,7 @@
         <v>67</v>
       </c>
       <c r="C62" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -2664,7 +2664,7 @@
         <v>68</v>
       </c>
       <c r="C63" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -2675,7 +2675,7 @@
         <v>69</v>
       </c>
       <c r="C64" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
@@ -2686,7 +2686,7 @@
         <v>70</v>
       </c>
       <c r="C65" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -2697,7 +2697,7 @@
         <v>71</v>
       </c>
       <c r="C66" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -2708,7 +2708,7 @@
         <v>72</v>
       </c>
       <c r="C67" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -2719,7 +2719,7 @@
         <v>73</v>
       </c>
       <c r="C68" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -2730,7 +2730,7 @@
         <v>74</v>
       </c>
       <c r="C69" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -2741,7 +2741,7 @@
         <v>75</v>
       </c>
       <c r="C70" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -2752,7 +2752,7 @@
         <v>76</v>
       </c>
       <c r="C71" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -2763,7 +2763,7 @@
         <v>77</v>
       </c>
       <c r="C72" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -2774,7 +2774,7 @@
         <v>78</v>
       </c>
       <c r="C73" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -2785,7 +2785,7 @@
         <v>79</v>
       </c>
       <c r="C74" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -2796,7 +2796,7 @@
         <v>80</v>
       </c>
       <c r="C75" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -2829,7 +2829,7 @@
         <v>83</v>
       </c>
       <c r="C78" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
@@ -2840,7 +2840,7 @@
         <v>85</v>
       </c>
       <c r="C79" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -2851,7 +2851,7 @@
         <v>86</v>
       </c>
       <c r="C80" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -2862,7 +2862,7 @@
         <v>87</v>
       </c>
       <c r="C81" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -2873,7 +2873,7 @@
         <v>88</v>
       </c>
       <c r="C82" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -2884,7 +2884,7 @@
         <v>89</v>
       </c>
       <c r="C83" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -2895,7 +2895,7 @@
         <v>90</v>
       </c>
       <c r="C84" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -2906,7 +2906,7 @@
         <v>91</v>
       </c>
       <c r="C85" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -2917,7 +2917,7 @@
         <v>92</v>
       </c>
       <c r="C86" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -2928,7 +2928,7 @@
         <v>93</v>
       </c>
       <c r="C87" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -2939,7 +2939,7 @@
         <v>94</v>
       </c>
       <c r="C88" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -2950,7 +2950,7 @@
         <v>95</v>
       </c>
       <c r="C89" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -2961,7 +2961,7 @@
         <v>96</v>
       </c>
       <c r="C90" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -2972,7 +2972,7 @@
         <v>97</v>
       </c>
       <c r="C91" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -2983,7 +2983,7 @@
         <v>98</v>
       </c>
       <c r="C92" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -2994,7 +2994,7 @@
         <v>99</v>
       </c>
       <c r="C93" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -3005,7 +3005,7 @@
         <v>100</v>
       </c>
       <c r="C94" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -3016,7 +3016,7 @@
         <v>101</v>
       </c>
       <c r="C95" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -3027,7 +3027,7 @@
         <v>102</v>
       </c>
       <c r="C96" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -3038,7 +3038,7 @@
         <v>103</v>
       </c>
       <c r="C97" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -3049,7 +3049,7 @@
         <v>104</v>
       </c>
       <c r="C98" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -3060,7 +3060,7 @@
         <v>105</v>
       </c>
       <c r="C99" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -3071,7 +3071,7 @@
         <v>106</v>
       </c>
       <c r="C100" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -3082,7 +3082,7 @@
         <v>107</v>
       </c>
       <c r="C101" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -3093,7 +3093,7 @@
         <v>108</v>
       </c>
       <c r="C102" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -3104,7 +3104,7 @@
         <v>109</v>
       </c>
       <c r="C103" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
@@ -3115,7 +3115,7 @@
         <v>111</v>
       </c>
       <c r="C104" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
@@ -3126,7 +3126,7 @@
         <v>112</v>
       </c>
       <c r="C105" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -3137,7 +3137,7 @@
         <v>113</v>
       </c>
       <c r="C106" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -3148,7 +3148,7 @@
         <v>114</v>
       </c>
       <c r="C107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -3159,7 +3159,7 @@
         <v>115</v>
       </c>
       <c r="C108" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -3170,7 +3170,7 @@
         <v>116</v>
       </c>
       <c r="C109" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -3181,7 +3181,7 @@
         <v>117</v>
       </c>
       <c r="C110" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -3192,7 +3192,7 @@
         <v>118</v>
       </c>
       <c r="C111" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -3203,7 +3203,7 @@
         <v>119</v>
       </c>
       <c r="C112" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
@@ -3214,7 +3214,7 @@
         <v>120</v>
       </c>
       <c r="C113" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -3225,7 +3225,7 @@
         <v>121</v>
       </c>
       <c r="C114" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -3236,7 +3236,7 @@
         <v>122</v>
       </c>
       <c r="C115" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
@@ -3247,7 +3247,7 @@
         <v>123</v>
       </c>
       <c r="C116" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -3258,7 +3258,7 @@
         <v>124</v>
       </c>
       <c r="C117" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -3269,7 +3269,7 @@
         <v>125</v>
       </c>
       <c r="C118" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -3280,7 +3280,7 @@
         <v>126</v>
       </c>
       <c r="C119" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -3291,7 +3291,7 @@
         <v>127</v>
       </c>
       <c r="C120" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -3302,7 +3302,7 @@
         <v>128</v>
       </c>
       <c r="C121" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -3313,7 +3313,7 @@
         <v>129</v>
       </c>
       <c r="C122" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -3324,7 +3324,7 @@
         <v>130</v>
       </c>
       <c r="C123" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -3335,7 +3335,7 @@
         <v>131</v>
       </c>
       <c r="C124" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -3346,7 +3346,7 @@
         <v>132</v>
       </c>
       <c r="C125" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -3357,7 +3357,7 @@
         <v>133</v>
       </c>
       <c r="C126" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -3368,7 +3368,7 @@
         <v>134</v>
       </c>
       <c r="C127" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -3379,7 +3379,7 @@
         <v>135</v>
       </c>
       <c r="C128" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -3390,7 +3390,7 @@
         <v>136</v>
       </c>
       <c r="C129" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -3401,7 +3401,7 @@
         <v>137</v>
       </c>
       <c r="C130" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -3412,7 +3412,7 @@
         <v>138</v>
       </c>
       <c r="C131" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -3423,7 +3423,7 @@
         <v>139</v>
       </c>
       <c r="C132" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
@@ -3434,7 +3434,7 @@
         <v>140</v>
       </c>
       <c r="C133" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -3445,7 +3445,7 @@
         <v>141</v>
       </c>
       <c r="C134" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -3456,7 +3456,7 @@
         <v>142</v>
       </c>
       <c r="C135" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -3467,7 +3467,7 @@
         <v>143</v>
       </c>
       <c r="C136" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -3478,7 +3478,7 @@
         <v>144</v>
       </c>
       <c r="C137" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -3489,7 +3489,7 @@
         <v>146</v>
       </c>
       <c r="C138" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -3500,7 +3500,7 @@
         <v>147</v>
       </c>
       <c r="C139" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -3511,7 +3511,7 @@
         <v>148</v>
       </c>
       <c r="C140" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -3522,7 +3522,7 @@
         <v>149</v>
       </c>
       <c r="C141" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -3533,7 +3533,7 @@
         <v>150</v>
       </c>
       <c r="C142" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -3544,7 +3544,7 @@
         <v>151</v>
       </c>
       <c r="C143" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -3555,7 +3555,7 @@
         <v>152</v>
       </c>
       <c r="C144" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -3566,7 +3566,7 @@
         <v>153</v>
       </c>
       <c r="C145" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -3577,7 +3577,7 @@
         <v>154</v>
       </c>
       <c r="C146" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
@@ -3588,7 +3588,7 @@
         <v>155</v>
       </c>
       <c r="C147" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -3599,7 +3599,7 @@
         <v>156</v>
       </c>
       <c r="C148" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -3610,7 +3610,7 @@
         <v>157</v>
       </c>
       <c r="C149" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -3621,7 +3621,7 @@
         <v>158</v>
       </c>
       <c r="C150" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -3632,7 +3632,7 @@
         <v>159</v>
       </c>
       <c r="C151" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -3643,7 +3643,7 @@
         <v>160</v>
       </c>
       <c r="C152" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -3654,7 +3654,7 @@
         <v>161</v>
       </c>
       <c r="C153" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -3665,7 +3665,7 @@
         <v>162</v>
       </c>
       <c r="C154" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -3676,7 +3676,7 @@
         <v>163</v>
       </c>
       <c r="C155" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -3687,7 +3687,7 @@
         <v>164</v>
       </c>
       <c r="C156" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -3698,7 +3698,7 @@
         <v>165</v>
       </c>
       <c r="C157" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -3709,7 +3709,7 @@
         <v>166</v>
       </c>
       <c r="C158" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -3720,7 +3720,7 @@
         <v>167</v>
       </c>
       <c r="C159" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
@@ -3731,7 +3731,7 @@
         <v>168</v>
       </c>
       <c r="C160" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
@@ -3742,7 +3742,7 @@
         <v>169</v>
       </c>
       <c r="C161" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
@@ -3753,7 +3753,7 @@
         <v>170</v>
       </c>
       <c r="C162" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
@@ -3764,7 +3764,7 @@
         <v>171</v>
       </c>
       <c r="C163" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
@@ -3775,7 +3775,7 @@
         <v>172</v>
       </c>
       <c r="C164" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
@@ -3786,7 +3786,7 @@
         <v>173</v>
       </c>
       <c r="C165" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
@@ -3797,7 +3797,7 @@
         <v>174</v>
       </c>
       <c r="C166" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
@@ -3808,7 +3808,7 @@
         <v>175</v>
       </c>
       <c r="C167" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
@@ -3819,7 +3819,7 @@
         <v>176</v>
       </c>
       <c r="C168" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
@@ -3830,7 +3830,7 @@
         <v>177</v>
       </c>
       <c r="C169" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
@@ -3841,7 +3841,7 @@
         <v>178</v>
       </c>
       <c r="C170" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.2">
@@ -3852,7 +3852,7 @@
         <v>179</v>
       </c>
       <c r="C171" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.2">
@@ -3863,7 +3863,7 @@
         <v>180</v>
       </c>
       <c r="C172" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.2">
@@ -3874,7 +3874,7 @@
         <v>181</v>
       </c>
       <c r="C173" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.2">
@@ -3885,7 +3885,7 @@
         <v>182</v>
       </c>
       <c r="C174" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
@@ -3896,7 +3896,7 @@
         <v>183</v>
       </c>
       <c r="C175" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
@@ -3907,7 +3907,7 @@
         <v>184</v>
       </c>
       <c r="C176" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
@@ -3918,7 +3918,7 @@
         <v>185</v>
       </c>
       <c r="C177" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.2">
@@ -3929,7 +3929,7 @@
         <v>186</v>
       </c>
       <c r="C178" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.2">
@@ -3940,7 +3940,7 @@
         <v>187</v>
       </c>
       <c r="C179" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.2">
@@ -3951,7 +3951,7 @@
         <v>188</v>
       </c>
       <c r="C180" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.2">
@@ -3962,7 +3962,7 @@
         <v>189</v>
       </c>
       <c r="C181" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.2">
@@ -3973,7 +3973,7 @@
         <v>190</v>
       </c>
       <c r="C182" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.2">
@@ -3984,7 +3984,7 @@
         <v>191</v>
       </c>
       <c r="C183" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.2">
@@ -3995,7 +3995,7 @@
         <v>192</v>
       </c>
       <c r="C184" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.2">
@@ -4006,7 +4006,7 @@
         <v>193</v>
       </c>
       <c r="C185" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.2">
@@ -4017,7 +4017,7 @@
         <v>194</v>
       </c>
       <c r="C186" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.2">
@@ -4028,7 +4028,7 @@
         <v>195</v>
       </c>
       <c r="C187" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.2">
@@ -4039,7 +4039,7 @@
         <v>196</v>
       </c>
       <c r="C188" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.2">
@@ -4050,7 +4050,7 @@
         <v>197</v>
       </c>
       <c r="C189" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.2">
@@ -4061,7 +4061,7 @@
         <v>198</v>
       </c>
       <c r="C190" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.2">
@@ -4072,7 +4072,7 @@
         <v>199</v>
       </c>
       <c r="C191" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.2">
@@ -4083,7 +4083,7 @@
         <v>200</v>
       </c>
       <c r="C192" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.2">
@@ -4094,7 +4094,7 @@
         <v>201</v>
       </c>
       <c r="C193" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.2">
@@ -4105,7 +4105,7 @@
         <v>202</v>
       </c>
       <c r="C194" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.2">
@@ -4116,7 +4116,7 @@
         <v>203</v>
       </c>
       <c r="C195" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.2">
@@ -4127,7 +4127,7 @@
         <v>204</v>
       </c>
       <c r="C196" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.2">
@@ -4138,7 +4138,7 @@
         <v>205</v>
       </c>
       <c r="C197" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.2">
@@ -4149,7 +4149,7 @@
         <v>206</v>
       </c>
       <c r="C198" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.2">
@@ -4160,7 +4160,7 @@
         <v>208</v>
       </c>
       <c r="C199" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.2">
@@ -4171,7 +4171,7 @@
         <v>209</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.2">
@@ -4182,7 +4182,7 @@
         <v>210</v>
       </c>
       <c r="C201" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.2">
@@ -4193,7 +4193,7 @@
         <v>211</v>
       </c>
       <c r="C202" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.2">
@@ -4204,7 +4204,7 @@
         <v>212</v>
       </c>
       <c r="C203" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.2">
@@ -4215,7 +4215,7 @@
         <v>213</v>
       </c>
       <c r="C204" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.2">
@@ -4226,7 +4226,7 @@
         <v>214</v>
       </c>
       <c r="C205" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.2">
@@ -4237,7 +4237,7 @@
         <v>215</v>
       </c>
       <c r="C206" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.2">
@@ -4248,7 +4248,7 @@
         <v>216</v>
       </c>
       <c r="C207" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.2">
@@ -4281,7 +4281,7 @@
         <v>219</v>
       </c>
       <c r="C210" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.2">
@@ -4292,7 +4292,7 @@
         <v>220</v>
       </c>
       <c r="C211" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.2">
@@ -4303,7 +4303,7 @@
         <v>221</v>
       </c>
       <c r="C212" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.2">
@@ -4314,7 +4314,7 @@
         <v>222</v>
       </c>
       <c r="C213" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.2">
@@ -4325,7 +4325,7 @@
         <v>223</v>
       </c>
       <c r="C214" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.2">
@@ -4336,7 +4336,7 @@
         <v>224</v>
       </c>
       <c r="C215" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.2">
@@ -4347,7 +4347,7 @@
         <v>225</v>
       </c>
       <c r="C216" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.2">
@@ -4369,7 +4369,7 @@
         <v>227</v>
       </c>
       <c r="C218" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.2">
@@ -4380,7 +4380,7 @@
         <v>228</v>
       </c>
       <c r="C219" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.2">
@@ -4391,7 +4391,7 @@
         <v>229</v>
       </c>
       <c r="C220" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.2">
@@ -4402,7 +4402,7 @@
         <v>230</v>
       </c>
       <c r="C221" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.2">
@@ -4413,7 +4413,7 @@
         <v>231</v>
       </c>
       <c r="C222" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.2">
@@ -4589,7 +4589,7 @@
         <v>247</v>
       </c>
       <c r="C238" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.2">
@@ -4600,7 +4600,7 @@
         <v>248</v>
       </c>
       <c r="C239" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.2">
@@ -4611,7 +4611,7 @@
         <v>249</v>
       </c>
       <c r="C240" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.2">
@@ -4622,7 +4622,7 @@
         <v>250</v>
       </c>
       <c r="C241" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.2">
@@ -4633,7 +4633,7 @@
         <v>251</v>
       </c>
       <c r="C242" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.2">
@@ -4677,7 +4677,7 @@
         <v>255</v>
       </c>
       <c r="C246" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.2">
@@ -4732,7 +4732,7 @@
         <v>260</v>
       </c>
       <c r="C251" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.2">
@@ -4743,7 +4743,7 @@
         <v>261</v>
       </c>
       <c r="C252" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.2">
@@ -4787,7 +4787,7 @@
         <v>265</v>
       </c>
       <c r="C256" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.2">
@@ -4798,7 +4798,7 @@
         <v>266</v>
       </c>
       <c r="C257" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.2">
@@ -4820,7 +4820,7 @@
         <v>269</v>
       </c>
       <c r="C259" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.2">
@@ -4831,7 +4831,7 @@
         <v>270</v>
       </c>
       <c r="C260" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.2">
@@ -4842,7 +4842,7 @@
         <v>271</v>
       </c>
       <c r="C261" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.2">
@@ -5007,7 +5007,7 @@
         <v>286</v>
       </c>
       <c r="C276" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.2">
@@ -5018,7 +5018,7 @@
         <v>287</v>
       </c>
       <c r="C277" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.2">
@@ -5029,7 +5029,7 @@
         <v>288</v>
       </c>
       <c r="C278" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.2">
@@ -5040,7 +5040,7 @@
         <v>289</v>
       </c>
       <c r="C279" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.2">
@@ -5051,7 +5051,7 @@
         <v>290</v>
       </c>
       <c r="C280" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.2">
@@ -5062,7 +5062,7 @@
         <v>291</v>
       </c>
       <c r="C281" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.2">
@@ -5073,7 +5073,7 @@
         <v>292</v>
       </c>
       <c r="C282" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.2">
@@ -5084,7 +5084,7 @@
         <v>293</v>
       </c>
       <c r="C283" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.2">
@@ -5095,7 +5095,7 @@
         <v>294</v>
       </c>
       <c r="C284" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.2">
@@ -5106,7 +5106,7 @@
         <v>295</v>
       </c>
       <c r="C285" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.2">
@@ -5117,7 +5117,7 @@
         <v>296</v>
       </c>
       <c r="C286" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.2">
@@ -5128,7 +5128,7 @@
         <v>297</v>
       </c>
       <c r="C287" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.2">
@@ -5139,7 +5139,7 @@
         <v>298</v>
       </c>
       <c r="C288" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.2">
@@ -5150,7 +5150,7 @@
         <v>299</v>
       </c>
       <c r="C289" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.2">
@@ -5161,7 +5161,7 @@
         <v>300</v>
       </c>
       <c r="C290" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.2">
@@ -5172,7 +5172,7 @@
         <v>301</v>
       </c>
       <c r="C291" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.2">
@@ -5183,7 +5183,7 @@
         <v>302</v>
       </c>
       <c r="C292" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.2">
@@ -5205,7 +5205,7 @@
         <v>304</v>
       </c>
       <c r="C294" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.2">
@@ -5315,7 +5315,7 @@
         <v>314</v>
       </c>
       <c r="C304" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.2">
@@ -5326,7 +5326,7 @@
         <v>315</v>
       </c>
       <c r="C305" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.2">
@@ -5337,7 +5337,7 @@
         <v>316</v>
       </c>
       <c r="C306" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.2">
@@ -5348,7 +5348,7 @@
         <v>317</v>
       </c>
       <c r="C307" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.2">
@@ -5359,7 +5359,7 @@
         <v>318</v>
       </c>
       <c r="C308" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.2">
@@ -5370,7 +5370,7 @@
         <v>319</v>
       </c>
       <c r="C309" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.2">
@@ -5381,7 +5381,7 @@
         <v>320</v>
       </c>
       <c r="C310" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.2">
@@ -5392,7 +5392,7 @@
         <v>321</v>
       </c>
       <c r="C311" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.2">
@@ -5403,7 +5403,7 @@
         <v>322</v>
       </c>
       <c r="C312" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.2">
@@ -5414,7 +5414,7 @@
         <v>323</v>
       </c>
       <c r="C313" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.2">
@@ -5425,7 +5425,7 @@
         <v>324</v>
       </c>
       <c r="C314" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.2">
@@ -5436,7 +5436,7 @@
         <v>325</v>
       </c>
       <c r="C315" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.2">
@@ -5447,7 +5447,7 @@
         <v>326</v>
       </c>
       <c r="C316" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.2">
@@ -5458,7 +5458,7 @@
         <v>327</v>
       </c>
       <c r="C317" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.2">
@@ -5469,7 +5469,7 @@
         <v>328</v>
       </c>
       <c r="C318" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.2">
@@ -5480,7 +5480,7 @@
         <v>329</v>
       </c>
       <c r="C319" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.2">
@@ -5491,7 +5491,7 @@
         <v>330</v>
       </c>
       <c r="C320" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.2">
@@ -5502,7 +5502,7 @@
         <v>331</v>
       </c>
       <c r="C321" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.2">
@@ -5513,7 +5513,7 @@
         <v>332</v>
       </c>
       <c r="C322" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.2">
@@ -5535,7 +5535,7 @@
         <v>334</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.2">
@@ -5546,7 +5546,7 @@
         <v>335</v>
       </c>
       <c r="C325" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.2">
@@ -5557,7 +5557,7 @@
         <v>336</v>
       </c>
       <c r="C326" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.2">
@@ -5568,7 +5568,7 @@
         <v>337</v>
       </c>
       <c r="C327" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.2">
@@ -5579,7 +5579,7 @@
         <v>338</v>
       </c>
       <c r="C328" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.2">
@@ -5590,7 +5590,7 @@
         <v>339</v>
       </c>
       <c r="C329" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.2">
@@ -5601,7 +5601,7 @@
         <v>340</v>
       </c>
       <c r="C330" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.2">
@@ -5612,7 +5612,7 @@
         <v>341</v>
       </c>
       <c r="C331" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.2">
@@ -5623,7 +5623,7 @@
         <v>342</v>
       </c>
       <c r="C332" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.2">
@@ -5634,7 +5634,7 @@
         <v>343</v>
       </c>
       <c r="C333" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.2">
@@ -5645,7 +5645,7 @@
         <v>344</v>
       </c>
       <c r="C334" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.2">
@@ -5656,7 +5656,7 @@
         <v>345</v>
       </c>
       <c r="C335" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.2">
@@ -5667,7 +5667,7 @@
         <v>346</v>
       </c>
       <c r="C336" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.2">
@@ -5678,7 +5678,7 @@
         <v>347</v>
       </c>
       <c r="C337" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.2">
@@ -5689,7 +5689,7 @@
         <v>348</v>
       </c>
       <c r="C338" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.2">
@@ -5700,7 +5700,7 @@
         <v>349</v>
       </c>
       <c r="C339" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.2">
@@ -5711,7 +5711,7 @@
         <v>350</v>
       </c>
       <c r="C340" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.2">
@@ -5722,7 +5722,7 @@
         <v>351</v>
       </c>
       <c r="C341" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.2">
@@ -5733,7 +5733,7 @@
         <v>352</v>
       </c>
       <c r="C342" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.2">
@@ -5744,7 +5744,7 @@
         <v>353</v>
       </c>
       <c r="C343" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.2">
@@ -5755,7 +5755,7 @@
         <v>354</v>
       </c>
       <c r="C344" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.2">
@@ -5766,7 +5766,7 @@
         <v>355</v>
       </c>
       <c r="C345" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.2">
@@ -5777,7 +5777,7 @@
         <v>356</v>
       </c>
       <c r="C346" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.2">
@@ -5788,7 +5788,7 @@
         <v>357</v>
       </c>
       <c r="C347" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.2">
@@ -5821,7 +5821,7 @@
         <v>360</v>
       </c>
       <c r="C350" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.2">
@@ -5832,7 +5832,7 @@
         <v>361</v>
       </c>
       <c r="C351" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.2">
@@ -5843,7 +5843,7 @@
         <v>362</v>
       </c>
       <c r="C352" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.2">
@@ -5854,7 +5854,7 @@
         <v>363</v>
       </c>
       <c r="C353" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.2">
@@ -5865,7 +5865,7 @@
         <v>364</v>
       </c>
       <c r="C354" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.2">
@@ -5876,7 +5876,7 @@
         <v>365</v>
       </c>
       <c r="C355" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="356" spans="1:3" x14ac:dyDescent="0.2">
@@ -5887,7 +5887,7 @@
         <v>366</v>
       </c>
       <c r="C356" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="357" spans="1:3" x14ac:dyDescent="0.2">
@@ -5898,7 +5898,7 @@
         <v>367</v>
       </c>
       <c r="C357" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="358" spans="1:3" x14ac:dyDescent="0.2">
@@ -5909,7 +5909,7 @@
         <v>368</v>
       </c>
       <c r="C358" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.2">
@@ -5920,7 +5920,7 @@
         <v>369</v>
       </c>
       <c r="C359" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.2">
@@ -5931,7 +5931,7 @@
         <v>370</v>
       </c>
       <c r="C360" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.2">
@@ -5942,7 +5942,7 @@
         <v>371</v>
       </c>
       <c r="C361" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.2">
@@ -5953,7 +5953,7 @@
         <v>372</v>
       </c>
       <c r="C362" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.2">
@@ -5964,7 +5964,7 @@
         <v>373</v>
       </c>
       <c r="C363" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.2">
@@ -5975,7 +5975,7 @@
         <v>374</v>
       </c>
       <c r="C364" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.2">
@@ -5986,7 +5986,7 @@
         <v>375</v>
       </c>
       <c r="C365" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.2">
@@ -5997,7 +5997,7 @@
         <v>376</v>
       </c>
       <c r="C366" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.2">
@@ -6008,7 +6008,7 @@
         <v>377</v>
       </c>
       <c r="C367" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.2">
@@ -6019,7 +6019,7 @@
         <v>378</v>
       </c>
       <c r="C368" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.2">
@@ -6030,7 +6030,7 @@
         <v>379</v>
       </c>
       <c r="C369" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.2">
@@ -6041,7 +6041,7 @@
         <v>380</v>
       </c>
       <c r="C370" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="371" spans="1:3" x14ac:dyDescent="0.2">
@@ -6052,7 +6052,7 @@
         <v>381</v>
       </c>
       <c r="C371" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="372" spans="1:3" x14ac:dyDescent="0.2">
@@ -6063,7 +6063,7 @@
         <v>382</v>
       </c>
       <c r="C372" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.2">
@@ -6074,7 +6074,7 @@
         <v>383</v>
       </c>
       <c r="C373" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="374" spans="1:3" x14ac:dyDescent="0.2">
@@ -6085,7 +6085,7 @@
         <v>384</v>
       </c>
       <c r="C374" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="375" spans="1:3" x14ac:dyDescent="0.2">
@@ -6096,7 +6096,7 @@
         <v>385</v>
       </c>
       <c r="C375" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="376" spans="1:3" x14ac:dyDescent="0.2">
@@ -6107,7 +6107,7 @@
         <v>386</v>
       </c>
       <c r="C376" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="377" spans="1:3" x14ac:dyDescent="0.2">
@@ -6118,7 +6118,7 @@
         <v>387</v>
       </c>
       <c r="C377" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="378" spans="1:3" x14ac:dyDescent="0.2">
@@ -6129,7 +6129,7 @@
         <v>388</v>
       </c>
       <c r="C378" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="379" spans="1:3" x14ac:dyDescent="0.2">
@@ -6140,7 +6140,7 @@
         <v>389</v>
       </c>
       <c r="C379" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.2">
@@ -6151,7 +6151,7 @@
         <v>390</v>
       </c>
       <c r="C380" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.2">
@@ -6162,7 +6162,7 @@
         <v>391</v>
       </c>
       <c r="C381" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="382" spans="1:3" x14ac:dyDescent="0.2">
@@ -6173,7 +6173,7 @@
         <v>392</v>
       </c>
       <c r="C382" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="383" spans="1:3" x14ac:dyDescent="0.2">
@@ -6184,7 +6184,7 @@
         <v>393</v>
       </c>
       <c r="C383" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.2">
@@ -6195,7 +6195,7 @@
         <v>394</v>
       </c>
       <c r="C384" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.2">
@@ -6206,7 +6206,7 @@
         <v>395</v>
       </c>
       <c r="C385" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.2">
@@ -6217,7 +6217,7 @@
         <v>396</v>
       </c>
       <c r="C386" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="387" spans="1:3" x14ac:dyDescent="0.2">
@@ -6228,7 +6228,7 @@
         <v>397</v>
       </c>
       <c r="C387" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.2">
@@ -6239,7 +6239,7 @@
         <v>398</v>
       </c>
       <c r="C388" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="389" spans="1:3" x14ac:dyDescent="0.2">
@@ -6250,7 +6250,7 @@
         <v>399</v>
       </c>
       <c r="C389" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="390" spans="1:3" x14ac:dyDescent="0.2">
@@ -6261,7 +6261,7 @@
         <v>400</v>
       </c>
       <c r="C390" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="391" spans="1:3" x14ac:dyDescent="0.2">
@@ -6272,7 +6272,7 @@
         <v>401</v>
       </c>
       <c r="C391" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.2">
@@ -6283,7 +6283,7 @@
         <v>402</v>
       </c>
       <c r="C392" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="393" spans="1:3" x14ac:dyDescent="0.2">
@@ -6327,7 +6327,7 @@
         <v>406</v>
       </c>
       <c r="C396" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="397" spans="1:3" x14ac:dyDescent="0.2">
@@ -6338,7 +6338,7 @@
         <v>407</v>
       </c>
       <c r="C397" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.2">
@@ -6349,7 +6349,7 @@
         <v>408</v>
       </c>
       <c r="C398" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.2">
@@ -6360,7 +6360,7 @@
         <v>409</v>
       </c>
       <c r="C399" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="400" spans="1:3" x14ac:dyDescent="0.2">
@@ -6371,7 +6371,7 @@
         <v>410</v>
       </c>
       <c r="C400" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="401" spans="1:3" x14ac:dyDescent="0.2">
@@ -6382,7 +6382,7 @@
         <v>411</v>
       </c>
       <c r="C401" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="402" spans="1:3" x14ac:dyDescent="0.2">
@@ -6393,7 +6393,7 @@
         <v>412</v>
       </c>
       <c r="C402" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="403" spans="1:3" x14ac:dyDescent="0.2">
@@ -6404,7 +6404,7 @@
         <v>413</v>
       </c>
       <c r="C403" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="404" spans="1:3" x14ac:dyDescent="0.2">
@@ -6415,7 +6415,7 @@
         <v>414</v>
       </c>
       <c r="C404" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="405" spans="1:3" x14ac:dyDescent="0.2">
@@ -6426,7 +6426,7 @@
         <v>415</v>
       </c>
       <c r="C405" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="406" spans="1:3" x14ac:dyDescent="0.2">
@@ -6437,7 +6437,7 @@
         <v>416</v>
       </c>
       <c r="C406" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="407" spans="1:3" x14ac:dyDescent="0.2">
@@ -6448,7 +6448,7 @@
         <v>417</v>
       </c>
       <c r="C407" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="408" spans="1:3" x14ac:dyDescent="0.2">
@@ -6459,7 +6459,7 @@
         <v>418</v>
       </c>
       <c r="C408" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="409" spans="1:3" x14ac:dyDescent="0.2">
@@ -6470,7 +6470,7 @@
         <v>419</v>
       </c>
       <c r="C409" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="410" spans="1:3" x14ac:dyDescent="0.2">
@@ -6481,7 +6481,7 @@
         <v>420</v>
       </c>
       <c r="C410" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="411" spans="1:3" x14ac:dyDescent="0.2">
@@ -6536,7 +6536,7 @@
         <v>425</v>
       </c>
       <c r="C415" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="416" spans="1:3" x14ac:dyDescent="0.2">
@@ -6547,7 +6547,7 @@
         <v>426</v>
       </c>
       <c r="C416" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.2">
@@ -6558,7 +6558,7 @@
         <v>427</v>
       </c>
       <c r="C417" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="418" spans="1:3" x14ac:dyDescent="0.2">
@@ -6569,7 +6569,7 @@
         <v>428</v>
       </c>
       <c r="C418" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="419" spans="1:3" x14ac:dyDescent="0.2">
@@ -6580,7 +6580,7 @@
         <v>429</v>
       </c>
       <c r="C419" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="420" spans="1:3" x14ac:dyDescent="0.2">
@@ -6591,7 +6591,7 @@
         <v>430</v>
       </c>
       <c r="C420" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="421" spans="1:3" x14ac:dyDescent="0.2">
@@ -6602,7 +6602,7 @@
         <v>431</v>
       </c>
       <c r="C421" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="422" spans="1:3" x14ac:dyDescent="0.2">
@@ -6613,7 +6613,7 @@
         <v>432</v>
       </c>
       <c r="C422" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="423" spans="1:3" x14ac:dyDescent="0.2">
@@ -6624,7 +6624,7 @@
         <v>433</v>
       </c>
       <c r="C423" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.2">
@@ -6635,7 +6635,7 @@
         <v>434</v>
       </c>
       <c r="C424" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="425" spans="1:3" x14ac:dyDescent="0.2">
@@ -6646,7 +6646,7 @@
         <v>435</v>
       </c>
       <c r="C425" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.2">
@@ -6657,7 +6657,7 @@
         <v>436</v>
       </c>
       <c r="C426" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="427" spans="1:3" x14ac:dyDescent="0.2">
@@ -6668,7 +6668,7 @@
         <v>437</v>
       </c>
       <c r="C427" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="428" spans="1:3" x14ac:dyDescent="0.2">
@@ -6679,7 +6679,7 @@
         <v>438</v>
       </c>
       <c r="C428" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="429" spans="1:3" x14ac:dyDescent="0.2">
@@ -6690,7 +6690,7 @@
         <v>439</v>
       </c>
       <c r="C429" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="430" spans="1:3" x14ac:dyDescent="0.2">
@@ -6701,7 +6701,7 @@
         <v>440</v>
       </c>
       <c r="C430" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="431" spans="1:3" x14ac:dyDescent="0.2">
@@ -6712,7 +6712,7 @@
         <v>441</v>
       </c>
       <c r="C431" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="432" spans="1:3" x14ac:dyDescent="0.2">
@@ -6723,7 +6723,7 @@
         <v>442</v>
       </c>
       <c r="C432" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="433" spans="1:3" x14ac:dyDescent="0.2">
@@ -6734,7 +6734,7 @@
         <v>443</v>
       </c>
       <c r="C433" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="434" spans="1:3" x14ac:dyDescent="0.2">
@@ -6745,7 +6745,7 @@
         <v>444</v>
       </c>
       <c r="C434" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="435" spans="1:3" x14ac:dyDescent="0.2">
@@ -6756,7 +6756,7 @@
         <v>445</v>
       </c>
       <c r="C435" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="436" spans="1:3" x14ac:dyDescent="0.2">
@@ -6767,7 +6767,7 @@
         <v>446</v>
       </c>
       <c r="C436" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="437" spans="1:3" x14ac:dyDescent="0.2">
@@ -6778,7 +6778,7 @@
         <v>447</v>
       </c>
       <c r="C437" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.2">
@@ -6789,7 +6789,7 @@
         <v>448</v>
       </c>
       <c r="C438" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.2">
@@ -6800,7 +6800,7 @@
         <v>449</v>
       </c>
       <c r="C439" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="440" spans="1:3" x14ac:dyDescent="0.2">
@@ -6811,7 +6811,7 @@
         <v>450</v>
       </c>
       <c r="C440" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="441" spans="1:3" x14ac:dyDescent="0.2">
@@ -6822,7 +6822,7 @@
         <v>451</v>
       </c>
       <c r="C441" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.2">
@@ -6833,7 +6833,7 @@
         <v>452</v>
       </c>
       <c r="C442" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="443" spans="1:3" x14ac:dyDescent="0.2">
@@ -6844,7 +6844,7 @@
         <v>453</v>
       </c>
       <c r="C443" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="444" spans="1:3" x14ac:dyDescent="0.2">
@@ -6855,7 +6855,7 @@
         <v>454</v>
       </c>
       <c r="C444" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="445" spans="1:3" x14ac:dyDescent="0.2">
@@ -6866,7 +6866,7 @@
         <v>455</v>
       </c>
       <c r="C445" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="446" spans="1:3" x14ac:dyDescent="0.2">
@@ -6877,7 +6877,7 @@
         <v>456</v>
       </c>
       <c r="C446" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.2">
@@ -6888,7 +6888,7 @@
         <v>457</v>
       </c>
       <c r="C447" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="448" spans="1:3" x14ac:dyDescent="0.2">
@@ -6899,7 +6899,7 @@
         <v>458</v>
       </c>
       <c r="C448" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="449" spans="1:3" x14ac:dyDescent="0.2">
@@ -6910,7 +6910,7 @@
         <v>459</v>
       </c>
       <c r="C449" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="450" spans="1:3" x14ac:dyDescent="0.2">
@@ -6921,7 +6921,7 @@
         <v>460</v>
       </c>
       <c r="C450" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.2">
@@ -6932,7 +6932,7 @@
         <v>461</v>
       </c>
       <c r="C451" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.2">
@@ -6943,7 +6943,7 @@
         <v>462</v>
       </c>
       <c r="C452" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.2">
@@ -6954,7 +6954,7 @@
         <v>463</v>
       </c>
       <c r="C453" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="454" spans="1:3" x14ac:dyDescent="0.2">
@@ -6965,7 +6965,7 @@
         <v>464</v>
       </c>
       <c r="C454" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.2">
@@ -6976,7 +6976,7 @@
         <v>465</v>
       </c>
       <c r="C455" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.2">
@@ -6987,7 +6987,7 @@
         <v>466</v>
       </c>
       <c r="C456" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.2">
@@ -6998,7 +6998,7 @@
         <v>467</v>
       </c>
       <c r="C457" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="458" spans="1:3" x14ac:dyDescent="0.2">
@@ -7009,7 +7009,7 @@
         <v>468</v>
       </c>
       <c r="C458" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="459" spans="1:3" x14ac:dyDescent="0.2">
@@ -7020,7 +7020,7 @@
         <v>469</v>
       </c>
       <c r="C459" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.2">
@@ -7031,7 +7031,7 @@
         <v>470</v>
       </c>
       <c r="C460" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="461" spans="1:3" x14ac:dyDescent="0.2">
@@ -7042,7 +7042,7 @@
         <v>471</v>
       </c>
       <c r="C461" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="462" spans="1:3" x14ac:dyDescent="0.2">
@@ -7053,7 +7053,7 @@
         <v>472</v>
       </c>
       <c r="C462" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="463" spans="1:3" x14ac:dyDescent="0.2">
@@ -7064,7 +7064,7 @@
         <v>473</v>
       </c>
       <c r="C463" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="464" spans="1:3" x14ac:dyDescent="0.2">
@@ -7075,7 +7075,7 @@
         <v>474</v>
       </c>
       <c r="C464" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.2">
@@ -7086,7 +7086,7 @@
         <v>475</v>
       </c>
       <c r="C465" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.2">
@@ -7097,7 +7097,7 @@
         <v>476</v>
       </c>
       <c r="C466" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.2">
@@ -7108,7 +7108,7 @@
         <v>477</v>
       </c>
       <c r="C467" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.2">
@@ -7119,7 +7119,7 @@
         <v>478</v>
       </c>
       <c r="C468" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.2">
@@ -7130,7 +7130,7 @@
         <v>479</v>
       </c>
       <c r="C469" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="470" spans="1:3" x14ac:dyDescent="0.2">
@@ -7141,7 +7141,7 @@
         <v>480</v>
       </c>
       <c r="C470" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="471" spans="1:3" x14ac:dyDescent="0.2">
@@ -7152,7 +7152,7 @@
         <v>481</v>
       </c>
       <c r="C471" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.2">
@@ -7163,7 +7163,7 @@
         <v>482</v>
       </c>
       <c r="C472" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.2">
@@ -7174,7 +7174,7 @@
         <v>483</v>
       </c>
       <c r="C473" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.2">
@@ -7185,7 +7185,7 @@
         <v>484</v>
       </c>
       <c r="C474" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.2">
@@ -7196,7 +7196,7 @@
         <v>485</v>
       </c>
       <c r="C475" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.2">
@@ -7207,7 +7207,7 @@
         <v>486</v>
       </c>
       <c r="C476" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.2">
@@ -7218,7 +7218,7 @@
         <v>487</v>
       </c>
       <c r="C477" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="478" spans="1:3" x14ac:dyDescent="0.2">
@@ -7229,7 +7229,7 @@
         <v>488</v>
       </c>
       <c r="C478" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="479" spans="1:3" x14ac:dyDescent="0.2">
@@ -7240,7 +7240,7 @@
         <v>489</v>
       </c>
       <c r="C479" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="480" spans="1:3" x14ac:dyDescent="0.2">
@@ -7251,7 +7251,7 @@
         <v>490</v>
       </c>
       <c r="C480" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.2">
@@ -7262,7 +7262,7 @@
         <v>491</v>
       </c>
       <c r="C481" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.2">
@@ -7273,7 +7273,7 @@
         <v>492</v>
       </c>
       <c r="C482" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="483" spans="1:3" x14ac:dyDescent="0.2">
@@ -7284,7 +7284,7 @@
         <v>493</v>
       </c>
       <c r="C483" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.2">
@@ -7295,7 +7295,7 @@
         <v>494</v>
       </c>
       <c r="C484" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.2">
@@ -7306,7 +7306,7 @@
         <v>495</v>
       </c>
       <c r="C485" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.2">
@@ -7317,7 +7317,7 @@
         <v>496</v>
       </c>
       <c r="C486" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.2">
@@ -7328,7 +7328,7 @@
         <v>497</v>
       </c>
       <c r="C487" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.2">
@@ -7339,7 +7339,7 @@
         <v>498</v>
       </c>
       <c r="C488" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.2">
@@ -7350,7 +7350,7 @@
         <v>499</v>
       </c>
       <c r="C489" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.2">
@@ -7361,7 +7361,7 @@
         <v>500</v>
       </c>
       <c r="C490" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.2">
@@ -7372,7 +7372,7 @@
         <v>501</v>
       </c>
       <c r="C491" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>